<commit_message>
Update training diagnostics and results for Llama model
- Updated figures for training diagnostics and perplexity in PDF and PNG formats.
- Revised LaTeX document to improve clarity and consistency in results presentation.
- Adjusted JSON data for open-ended uncertainty metrics, including new perplexity and distinct values.
- Enhanced Python scripts to incorporate autoregressive reference metrics for better comparison in results.
- Added new data points for training progression and adjusted the selection of global steps for analysis.
</commit_message>
<xml_diff>
--- a/iclr2027_submission/source_results/Results_training-progression-long32i-64i_20260923.xlsx
+++ b/iclr2027_submission/source_results/Results_training-progression-long32i-64i_20260923.xlsx
@@ -3113,8 +3113,14 @@
       <c r="P44" s="5" t="n">
         <v>5.334906578063965</v>
       </c>
-      <c r="Q44" s="8" t="n"/>
-      <c r="R44" s="8" t="n"/>
+      <c r="Q44" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R44" s="8" t="n">
+        <v>2.638597726821899</v>
+      </c>
       <c r="S44" s="8" t="n"/>
       <c r="T44" s="8" t="n"/>
       <c r="U44" s="8" t="n"/>
@@ -3133,27 +3139,37 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>10.72950077056885</v>
-      </c>
-      <c r="E45" s="5" t="n"/>
+        <v>11.69381046295166</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>12.16381454467773</v>
+      </c>
       <c r="F45" s="5" t="n">
-        <v>11.47562980651855</v>
-      </c>
-      <c r="G45" s="5" t="n"/>
+        <v>11.07769298553467</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>10.21605587005615</v>
+      </c>
       <c r="H45" s="5" t="n">
-        <v>10.27829837799072</v>
-      </c>
-      <c r="I45" s="5" t="n"/>
+        <v>10.07588672637939</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>9.757587432861328</v>
+      </c>
       <c r="J45" s="5" t="n">
-        <v>8.44993782043457</v>
-      </c>
-      <c r="K45" s="5" t="n"/>
+        <v>11.00800037384033</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>9.088900566101074</v>
+      </c>
       <c r="L45" s="5" t="n">
-        <v>9.874661445617676</v>
-      </c>
-      <c r="M45" s="5" t="n"/>
+        <v>9.759171485900879</v>
+      </c>
+      <c r="M45" s="5" t="n">
+        <v>10.43219089508057</v>
+      </c>
       <c r="N45" s="5" t="n">
-        <v>9.490921020507812</v>
+        <v>9.534310340881348</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -3163,8 +3179,14 @@
       <c r="P45" s="5" t="n">
         <v>4.065366268157959</v>
       </c>
-      <c r="Q45" s="8" t="n"/>
-      <c r="R45" s="8" t="n"/>
+      <c r="Q45" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R45" s="8" t="n">
+        <v>2.638597726821899</v>
+      </c>
       <c r="S45" s="8" t="n"/>
       <c r="T45" s="8" t="n"/>
       <c r="U45" s="8" t="n"/>
@@ -3213,8 +3235,14 @@
       <c r="P46" s="14" t="n">
         <v>2.794792175292969</v>
       </c>
-      <c r="Q46" s="8" t="n"/>
-      <c r="R46" s="8" t="n"/>
+      <c r="Q46" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R46" s="8" t="n">
+        <v>2.638597726821899</v>
+      </c>
       <c r="S46" s="8" t="n"/>
       <c r="T46" s="8" t="n"/>
       <c r="U46" s="8" t="n"/>
@@ -3418,8 +3446,14 @@
       <c r="P51" s="5" t="n">
         <v>0.4518068870489012</v>
       </c>
-      <c r="Q51" s="8" t="n"/>
-      <c r="R51" s="8" t="n"/>
+      <c r="Q51" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R51" s="8" t="n">
+        <v>0.620703125</v>
+      </c>
       <c r="S51" s="8" t="n"/>
       <c r="T51" s="8" t="n"/>
       <c r="U51" s="8" t="n"/>
@@ -3443,27 +3477,37 @@
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.4036814788479851</v>
-      </c>
-      <c r="E52" s="5" t="n"/>
+        <v>0.4770001857813828</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v>0.5036962743523382</v>
+      </c>
       <c r="F52" s="5" t="n">
-        <v>0.5183219930624684</v>
-      </c>
-      <c r="G52" s="5" t="n"/>
+        <v>0.4949032341102356</v>
+      </c>
+      <c r="G52" s="5" t="n">
+        <v>0.4603871065091548</v>
+      </c>
       <c r="H52" s="5" t="n">
-        <v>0.4928850947708592</v>
-      </c>
-      <c r="I52" s="5" t="n"/>
+        <v>0.4900945150578522</v>
+      </c>
+      <c r="I52" s="5" t="n">
+        <v>0.4761299096660723</v>
+      </c>
       <c r="J52" s="5" t="n">
-        <v>0.4267567054340076</v>
-      </c>
-      <c r="K52" s="5" t="n"/>
+        <v>0.5660157300756498</v>
+      </c>
+      <c r="K52" s="5" t="n">
+        <v>0.4829679223470319</v>
+      </c>
       <c r="L52" s="5" t="n">
-        <v>0.501915020026646</v>
-      </c>
-      <c r="M52" s="5" t="n"/>
+        <v>0.4940800474890126</v>
+      </c>
+      <c r="M52" s="5" t="n">
+        <v>0.5588273675088411</v>
+      </c>
       <c r="N52" s="5" t="n">
-        <v>0.5077240599008827</v>
+        <v>0.4961229208330553</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -3473,8 +3517,14 @@
       <c r="P52" s="5" t="n">
         <v>0.5137462150564513</v>
       </c>
-      <c r="Q52" s="8" t="n"/>
-      <c r="R52" s="8" t="n"/>
+      <c r="Q52" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R52" s="8" t="n">
+        <v>0.620703125</v>
+      </c>
       <c r="S52" s="8" t="n"/>
       <c r="T52" s="8" t="n"/>
       <c r="U52" s="8" t="n"/>
@@ -3511,8 +3561,14 @@
       <c r="P53" s="14" t="n">
         <v>0.5339673886917981</v>
       </c>
-      <c r="Q53" s="8" t="n"/>
-      <c r="R53" s="8" t="n"/>
+      <c r="Q53" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R53" s="8" t="n">
+        <v>0.620703125</v>
+      </c>
       <c r="S53" s="8" t="n"/>
       <c r="T53" s="8" t="n"/>
       <c r="U53" s="8" t="n"/>
@@ -3706,8 +3762,14 @@
       <c r="P58" s="5" t="n">
         <v>0.7458363992037593</v>
       </c>
-      <c r="Q58" s="8" t="n"/>
-      <c r="R58" s="8" t="n"/>
+      <c r="Q58" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R58" s="8" t="n">
+        <v>0.8956692913385826</v>
+      </c>
       <c r="S58" s="8" t="n"/>
       <c r="T58" s="8" t="n"/>
       <c r="U58" s="8" t="n"/>
@@ -3726,27 +3788,37 @@
         </is>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.6821036360128161</v>
-      </c>
-      <c r="E59" s="5" t="n"/>
+        <v>0.7653417136140228</v>
+      </c>
+      <c r="E59" s="5" t="n">
+        <v>0.8087142432097123</v>
+      </c>
       <c r="F59" s="5" t="n">
-        <v>0.8118560849225821</v>
-      </c>
-      <c r="G59" s="5" t="n"/>
+        <v>0.7868520256811472</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>0.7448636685412484</v>
+      </c>
       <c r="H59" s="5" t="n">
-        <v>0.7712423402838213</v>
-      </c>
-      <c r="I59" s="5" t="n"/>
+        <v>0.7818280329221895</v>
+      </c>
+      <c r="I59" s="5" t="n">
+        <v>0.7680126304153245</v>
+      </c>
       <c r="J59" s="5" t="n">
-        <v>0.7216139638297008</v>
-      </c>
-      <c r="K59" s="5" t="n"/>
+        <v>0.8465911235602921</v>
+      </c>
+      <c r="K59" s="5" t="n">
+        <v>0.7773631990335352</v>
+      </c>
       <c r="L59" s="5" t="n">
-        <v>0.789281943708992</v>
-      </c>
-      <c r="M59" s="5" t="n"/>
+        <v>0.7854051040450196</v>
+      </c>
+      <c r="M59" s="5" t="n">
+        <v>0.8381913301726476</v>
+      </c>
       <c r="N59" s="5" t="n">
-        <v>0.7821560718720321</v>
+        <v>0.7912437391323626</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -3756,8 +3828,14 @@
       <c r="P59" s="5" t="n">
         <v>0.8228125277351084</v>
       </c>
-      <c r="Q59" s="8" t="n"/>
-      <c r="R59" s="8" t="n"/>
+      <c r="Q59" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R59" s="8" t="n">
+        <v>0.8956692913385826</v>
+      </c>
       <c r="S59" s="8" t="n"/>
       <c r="T59" s="8" t="n"/>
       <c r="U59" s="8" t="n"/>
@@ -3794,8 +3872,14 @@
       <c r="P60" s="14" t="n">
         <v>0.8494491582491582</v>
       </c>
-      <c r="Q60" s="8" t="n"/>
-      <c r="R60" s="8" t="n"/>
+      <c r="Q60" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R60" s="8" t="n">
+        <v>0.8956692913385826</v>
+      </c>
       <c r="S60" s="8" t="n"/>
       <c r="T60" s="8" t="n"/>
       <c r="U60" s="8" t="n"/>
@@ -3985,8 +4069,14 @@
       <c r="P65" s="5" t="n">
         <v>0.8447467723417461</v>
       </c>
-      <c r="Q65" s="8" t="n"/>
-      <c r="R65" s="8" t="n"/>
+      <c r="Q65" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R65" s="8" t="n">
+        <v>0.954047619047619</v>
+      </c>
       <c r="S65" s="8" t="n"/>
       <c r="T65" s="8" t="n"/>
       <c r="U65" s="8" t="n"/>
@@ -4005,27 +4095,37 @@
         </is>
       </c>
       <c r="D66" s="5" t="n">
-        <v>0.80782224413182</v>
-      </c>
-      <c r="E66" s="5" t="n"/>
+        <v>0.8638053978946415</v>
+      </c>
+      <c r="E66" s="5" t="n">
+        <v>0.9064424200671979</v>
+      </c>
       <c r="F66" s="5" t="n">
-        <v>0.9035521513137563</v>
-      </c>
-      <c r="G66" s="5" t="n"/>
+        <v>0.8838037665060672</v>
+      </c>
+      <c r="G66" s="5" t="n">
+        <v>0.8523986307869598</v>
+      </c>
       <c r="H66" s="5" t="n">
-        <v>0.8697687993137726</v>
-      </c>
-      <c r="I66" s="5" t="n"/>
+        <v>0.8801325382828397</v>
+      </c>
+      <c r="I66" s="5" t="n">
+        <v>0.8735682715414933</v>
+      </c>
       <c r="J66" s="5" t="n">
-        <v>0.8370939114713054</v>
-      </c>
-      <c r="K66" s="5" t="n"/>
+        <v>0.9242393333892163</v>
+      </c>
+      <c r="K66" s="5" t="n">
+        <v>0.8778186678489756</v>
+      </c>
       <c r="L66" s="5" t="n">
-        <v>0.8874663373466863</v>
-      </c>
-      <c r="M66" s="5" t="n"/>
+        <v>0.8864254779840042</v>
+      </c>
+      <c r="M66" s="5" t="n">
+        <v>0.9232639157226578</v>
+      </c>
       <c r="N66" s="5" t="n">
-        <v>0.8777448656611037</v>
+        <v>0.8918719251653024</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -4035,8 +4135,14 @@
       <c r="P66" s="5" t="n">
         <v>0.9160808112597255</v>
       </c>
-      <c r="Q66" s="8" t="n"/>
-      <c r="R66" s="8" t="n"/>
+      <c r="Q66" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R66" s="8" t="n">
+        <v>0.954047619047619</v>
+      </c>
       <c r="S66" s="8" t="n"/>
       <c r="T66" s="8" t="n"/>
       <c r="U66" s="8" t="n"/>
@@ -4073,8 +4179,14 @@
       <c r="P67" s="14" t="n">
         <v>0.9334603282399547</v>
       </c>
-      <c r="Q67" s="8" t="n"/>
-      <c r="R67" s="8" t="n"/>
+      <c r="Q67" s="8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R67" s="8" t="n">
+        <v>0.954047619047619</v>
+      </c>
       <c r="S67" s="8" t="n"/>
       <c r="T67" s="8" t="n"/>
       <c r="U67" s="8" t="n"/>
@@ -6291,7 +6403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:P35"/>
+  <dimension ref="A3:R35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="24.83203125" bestFit="1" customWidth="1" style="33" min="2" max="2"/>
@@ -6449,6 +6561,14 @@
       <c r="P6" t="n">
         <v>5.334906578063965</v>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>2.638597726821899</v>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="33">
       <c r="B7" s="7" t="inlineStr">
@@ -6462,37 +6582,37 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>10.72950077056885</v>
+        <v>11.69381046295166</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>10.015</v>
+        <v>12.16381454467773</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>11.47562980651855</v>
+        <v>11.07769298553467</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>9.646000000000001</v>
+        <v>10.21605587005615</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>10.27829837799072</v>
+        <v>10.07588672637939</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>9.839</v>
+        <v>9.757587432861328</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>8.44993782043457</v>
+        <v>11.00800037384033</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>8.715999999999999</v>
+        <v>9.088900566101074</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>9.874661445617676</v>
+        <v>9.759171485900879</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>8.382</v>
+        <v>10.43219089508057</v>
       </c>
       <c r="N7" s="31" t="n">
-        <v>9.490921020507812</v>
+        <v>9.534310340881348</v>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
@@ -6501,6 +6621,14 @@
       </c>
       <c r="P7" t="n">
         <v>4.065366268157959</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>2.638597726821899</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="33">
@@ -6546,6 +6674,14 @@
       </c>
       <c r="P8" t="n">
         <v>2.794792175292969</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>2.638597726821899</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1" s="33">
@@ -6875,6 +7011,14 @@
       <c r="P19" t="n">
         <v>0.4518068870489012</v>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>0.620703125</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1" s="33">
       <c r="B20" s="7" t="n"/>
@@ -6884,27 +7028,37 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.4036814788479851</v>
-      </c>
-      <c r="E20" s="5" t="n"/>
+        <v>0.4770001857813828</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>0.5036962743523382</v>
+      </c>
       <c r="F20" s="5" t="n">
-        <v>0.5183219930624684</v>
-      </c>
-      <c r="G20" s="5" t="n"/>
+        <v>0.4949032341102356</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0.4603871065091548</v>
+      </c>
       <c r="H20" s="5" t="n">
-        <v>0.4928850947708592</v>
-      </c>
-      <c r="I20" s="5" t="n"/>
+        <v>0.4900945150578522</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>0.4761299096660723</v>
+      </c>
       <c r="J20" s="5" t="n">
-        <v>0.4267567054340076</v>
-      </c>
-      <c r="K20" s="5" t="n"/>
+        <v>0.5660157300756498</v>
+      </c>
+      <c r="K20" s="5" t="n">
+        <v>0.4829679223470319</v>
+      </c>
       <c r="L20" s="5" t="n">
-        <v>0.501915020026646</v>
-      </c>
-      <c r="M20" s="5" t="n"/>
+        <v>0.4940800474890126</v>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>0.5588273675088411</v>
+      </c>
       <c r="N20" s="31" t="n">
-        <v>0.5077240599008827</v>
+        <v>0.4961229208330553</v>
       </c>
       <c r="O20" s="5" t="inlineStr">
         <is>
@@ -6913,6 +7067,14 @@
       </c>
       <c r="P20" t="n">
         <v>0.5137462150564513</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>0.620703125</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="33">
@@ -6941,6 +7103,14 @@
       <c r="P21" t="n">
         <v>0.5339673886917981</v>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R21" t="n">
+        <v>0.620703125</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="33">
       <c r="A24" s="31" t="n"/>
@@ -7055,6 +7225,14 @@
       <c r="P26" t="n">
         <v>0.7458363992037593</v>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R26" t="n">
+        <v>0.8956692913385826</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="33">
       <c r="B27" s="7" t="n"/>
@@ -7064,27 +7242,37 @@
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.6821036360128161</v>
-      </c>
-      <c r="E27" s="5" t="n"/>
+        <v>0.7653417136140228</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.8087142432097123</v>
+      </c>
       <c r="F27" s="5" t="n">
-        <v>0.8118560849225821</v>
-      </c>
-      <c r="G27" s="5" t="n"/>
+        <v>0.7868520256811472</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.7448636685412484</v>
+      </c>
       <c r="H27" s="5" t="n">
-        <v>0.7712423402838213</v>
-      </c>
-      <c r="I27" s="5" t="n"/>
+        <v>0.7818280329221895</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0.7680126304153245</v>
+      </c>
       <c r="J27" s="5" t="n">
-        <v>0.7216139638297008</v>
-      </c>
-      <c r="K27" s="5" t="n"/>
+        <v>0.8465911235602921</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>0.7773631990335352</v>
+      </c>
       <c r="L27" s="5" t="n">
-        <v>0.789281943708992</v>
-      </c>
-      <c r="M27" s="5" t="n"/>
+        <v>0.7854051040450196</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>0.8381913301726476</v>
+      </c>
       <c r="N27" s="31" t="n">
-        <v>0.7821560718720321</v>
+        <v>0.7912437391323626</v>
       </c>
       <c r="O27" s="5" t="inlineStr">
         <is>
@@ -7093,6 +7281,14 @@
       </c>
       <c r="P27" t="n">
         <v>0.8228125277351084</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>0.8956692913385826</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1" s="33">
@@ -7121,6 +7317,14 @@
       <c r="P28" t="n">
         <v>0.8494491582491582</v>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R28" t="n">
+        <v>0.8956692913385826</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="33">
       <c r="A31" s="31" t="n"/>
@@ -7235,6 +7439,14 @@
       <c r="P33" t="n">
         <v>0.8447467723417461</v>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R33" t="n">
+        <v>0.954047619047619</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1" s="33">
       <c r="B34" s="7" t="n"/>
@@ -7244,27 +7456,37 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.80782224413182</v>
-      </c>
-      <c r="E34" s="5" t="n"/>
+        <v>0.8638053978946415</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>0.9064424200671979</v>
+      </c>
       <c r="F34" s="5" t="n">
-        <v>0.9035521513137563</v>
-      </c>
-      <c r="G34" s="5" t="n"/>
+        <v>0.8838037665060672</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0.8523986307869598</v>
+      </c>
       <c r="H34" s="5" t="n">
-        <v>0.8697687993137726</v>
-      </c>
-      <c r="I34" s="5" t="n"/>
+        <v>0.8801325382828397</v>
+      </c>
+      <c r="I34" s="5" t="n">
+        <v>0.8735682715414933</v>
+      </c>
       <c r="J34" s="5" t="n">
-        <v>0.8370939114713054</v>
-      </c>
-      <c r="K34" s="5" t="n"/>
+        <v>0.9242393333892163</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>0.8778186678489756</v>
+      </c>
       <c r="L34" s="5" t="n">
-        <v>0.8874663373466863</v>
-      </c>
-      <c r="M34" s="5" t="n"/>
+        <v>0.8864254779840042</v>
+      </c>
+      <c r="M34" s="5" t="n">
+        <v>0.9232639157226578</v>
+      </c>
       <c r="N34" s="31" t="n">
-        <v>0.8777448656611037</v>
+        <v>0.8918719251653024</v>
       </c>
       <c r="O34" s="5" t="inlineStr">
         <is>
@@ -7273,6 +7495,14 @@
       </c>
       <c r="P34" t="n">
         <v>0.9160808112597255</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R34" t="n">
+        <v>0.954047619047619</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="33">
@@ -7301,6 +7531,14 @@
       <c r="P35" t="n">
         <v>0.9334603282399547</v>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Llama 3.1 8B AR</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>0.954047619047619</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7401,7 +7639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B81"/>
+  <dimension ref="A1:B86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" style="33" min="1" max="1"/>
@@ -8190,7 +8428,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>20260922T182255.239456Z--colab-validation</t>
+          <t>20260923T190517.263478Z--colab-validation</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8440,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-09-22T19:31:40.697494+00:00</t>
+          <t>2026-09-23T20:08:05.344501+00:00</t>
         </is>
       </c>
     </row>
@@ -8214,7 +8452,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/validation/benchmark_runs/20260922T182255.239456Z--colab-validation/summary.json</t>
+          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/validation/benchmark_runs/20260923T190517.263478Z--colab-validation/summary.json</t>
         </is>
       </c>
     </row>
@@ -8226,7 +8464,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>1k, 10k, 20k, 30k, 40k, 50k</t>
+          <t>1k, 5k, 10k, 15k, 20k, 25k, 30k, 35k, 40k, 45k, 50k</t>
         </is>
       </c>
     </row>
@@ -8255,36 +8493,90 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Long-run validation-loss source</t>
+          <t>Autoregressive reference run ID</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/outputs/llama-3.1-8b-mask-long/metrics.jsonl</t>
+          <t>20260923T134029.046940Z--colab-validation</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Long-run validation-loss snapshot</t>
+          <t>Autoregressive reference model</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>steps 500--50000 in increments of 500</t>
+          <t>meta-llama/Llama-3.1-8B-Instruct</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>Autoregressive reference scored prompts</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Autoregressive reference perplexity</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2.638597726821899</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Autoregressive reference mean Distinct-1</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0.620703125</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Long-run validation-loss source</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/outputs/llama-3.1-8b-mask-long/metrics.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Long-run validation-loss snapshot</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>steps 500--50000 in increments of 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
           <t>Progression import timestamp UTC</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>2026-09-23T15:29:08.638544+00:00</t>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-09-23T20:12:06.859324+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update training diagnostics and results for ICLR 2027 submission
- Revised `RESULTS_NOTES.md` to reflect changes in llama training diagnostics and added details on targeted seed replication run.
- Updated `figure_data.json` with new perplexity and Distinct-1 values, increasing sample size to 100 prompts for various checkpoints.
- Modified `calculate_open_ended_uncertainty.py` and `import_progression_results.py` to reference the latest progression runs and include 128 NFE in selected steps.
- Replaced outdated progression run IDs in multiple scripts and JSON files.
- Updated binary figures for benchmark radar panels and llama training diagnostics.
</commit_message>
<xml_diff>
--- a/iclr2027_submission/source_results/Results_training-progression-long32i-64i_20260923.xlsx
+++ b/iclr2027_submission/source_results/Results_training-progression-long32i-64i_20260923.xlsx
@@ -3205,27 +3205,37 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>5.7954</v>
-      </c>
-      <c r="E46" s="5" t="n"/>
+        <v>6.043358325958252</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>5.753337860107422</v>
+      </c>
       <c r="F46" s="5" t="n">
-        <v>5.2868</v>
-      </c>
-      <c r="G46" s="5" t="n"/>
+        <v>5.449683666229248</v>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>5.394126892089844</v>
+      </c>
       <c r="H46" s="5" t="n">
-        <v>4.7627</v>
-      </c>
-      <c r="I46" s="5" t="n"/>
+        <v>4.890061378479004</v>
+      </c>
+      <c r="I46" s="5" t="n">
+        <v>5.126490116119385</v>
+      </c>
       <c r="J46" s="5" t="n">
-        <v>4.6642</v>
-      </c>
-      <c r="K46" s="5" t="n"/>
+        <v>5.103343963623047</v>
+      </c>
+      <c r="K46" s="5" t="n">
+        <v>4.802248001098633</v>
+      </c>
       <c r="L46" s="5" t="n">
-        <v>4.4202</v>
-      </c>
-      <c r="M46" s="5" t="n"/>
+        <v>5.045702934265137</v>
+      </c>
+      <c r="M46" s="5" t="n">
+        <v>5.248916149139404</v>
+      </c>
       <c r="N46" s="5" t="n">
-        <v>4.8757</v>
+        <v>4.829687595367432</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -3542,17 +3552,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="5" t="n"/>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="5" t="n"/>
-      <c r="K53" s="5" t="n"/>
-      <c r="L53" s="5" t="n"/>
-      <c r="M53" s="5" t="n"/>
-      <c r="N53" s="5" t="n"/>
+      <c r="D53" s="5" t="n">
+        <v>0.5054446859283357</v>
+      </c>
+      <c r="E53" s="5" t="n">
+        <v>0.519199366453035</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>0.5178086392366672</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>0.4954837457655661</v>
+      </c>
+      <c r="H53" s="5" t="n">
+        <v>0.511337848264892</v>
+      </c>
+      <c r="I53" s="5" t="n">
+        <v>0.50891858524168</v>
+      </c>
+      <c r="J53" s="5" t="n">
+        <v>0.5717420902235882</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>0.5275748647375792</v>
+      </c>
+      <c r="L53" s="5" t="n">
+        <v>0.5119562703885332</v>
+      </c>
+      <c r="M53" s="5" t="n">
+        <v>0.5843122972986872</v>
+      </c>
+      <c r="N53" s="5" t="n">
+        <v>0.5073863484216871</v>
+      </c>
       <c r="O53" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -3853,17 +3885,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D60" s="5" t="n"/>
-      <c r="E60" s="5" t="n"/>
-      <c r="F60" s="5" t="n"/>
-      <c r="G60" s="5" t="n"/>
-      <c r="H60" s="5" t="n"/>
-      <c r="I60" s="5" t="n"/>
-      <c r="J60" s="5" t="n"/>
-      <c r="K60" s="5" t="n"/>
-      <c r="L60" s="5" t="n"/>
-      <c r="M60" s="5" t="n"/>
-      <c r="N60" s="5" t="n"/>
+      <c r="D60" s="5" t="n">
+        <v>0.7830597621110132</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v>0.8064073298678864</v>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>0.7937104727462332</v>
+      </c>
+      <c r="G60" s="5" t="n">
+        <v>0.7627448026242314</v>
+      </c>
+      <c r="H60" s="5" t="n">
+        <v>0.8009410518420114</v>
+      </c>
+      <c r="I60" s="5" t="n">
+        <v>0.7909752895896033</v>
+      </c>
+      <c r="J60" s="5" t="n">
+        <v>0.8419165604351599</v>
+      </c>
+      <c r="K60" s="5" t="n">
+        <v>0.8160420765709792</v>
+      </c>
+      <c r="L60" s="5" t="n">
+        <v>0.798767023558475</v>
+      </c>
+      <c r="M60" s="5" t="n">
+        <v>0.8552598551268979</v>
+      </c>
+      <c r="N60" s="5" t="n">
+        <v>0.7923201582427839</v>
+      </c>
       <c r="O60" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -4160,17 +4214,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D67" s="5" t="n"/>
-      <c r="E67" s="5" t="n"/>
-      <c r="F67" s="5" t="n"/>
-      <c r="G67" s="5" t="n"/>
-      <c r="H67" s="5" t="n"/>
-      <c r="I67" s="5" t="n"/>
-      <c r="J67" s="5" t="n"/>
-      <c r="K67" s="5" t="n"/>
-      <c r="L67" s="5" t="n"/>
-      <c r="M67" s="5" t="n"/>
-      <c r="N67" s="5" t="n"/>
+      <c r="D67" s="5" t="n">
+        <v>0.8727189519854217</v>
+      </c>
+      <c r="E67" s="5" t="n">
+        <v>0.8991272440231518</v>
+      </c>
+      <c r="F67" s="5" t="n">
+        <v>0.8846654157733219</v>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>0.8559358721535252</v>
+      </c>
+      <c r="H67" s="5" t="n">
+        <v>0.8956816655050087</v>
+      </c>
+      <c r="I67" s="5" t="n">
+        <v>0.8853025773993753</v>
+      </c>
+      <c r="J67" s="5" t="n">
+        <v>0.9242696608846586</v>
+      </c>
+      <c r="K67" s="5" t="n">
+        <v>0.9041828997570535</v>
+      </c>
+      <c r="L67" s="5" t="n">
+        <v>0.8914650348851834</v>
+      </c>
+      <c r="M67" s="5" t="n">
+        <v>0.9318457286887116</v>
+      </c>
+      <c r="N67" s="5" t="n">
+        <v>0.8864252529499462</v>
+      </c>
       <c r="O67" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -6642,30 +6718,38 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
+      <c r="D8" s="5" t="n">
+        <v>6.043358325958252</v>
+      </c>
       <c r="E8" s="5" t="n">
-        <v>5.2868</v>
-      </c>
-      <c r="F8" s="5" t="n"/>
+        <v>5.753337860107422</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>5.449683666229248</v>
+      </c>
       <c r="G8" s="5" t="n">
-        <v>4.7627</v>
-      </c>
-      <c r="H8" s="5" t="n"/>
+        <v>5.394126892089844</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>4.890061378479004</v>
+      </c>
       <c r="I8" s="5" t="n">
-        <v>4.6642</v>
-      </c>
-      <c r="J8" s="5" t="n"/>
+        <v>5.126490116119385</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>5.103343963623047</v>
+      </c>
       <c r="K8" s="5" t="n">
-        <v>4.4202</v>
-      </c>
-      <c r="L8" s="5" t="n"/>
+        <v>4.802248001098633</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>5.045702934265137</v>
+      </c>
       <c r="M8" s="5" t="n">
-        <v>4.8757</v>
-      </c>
-      <c r="N8" s="31" t="inlineStr">
-        <is>
-          <t>LlaDa (128 it.)</t>
-        </is>
+        <v>5.248916149139404</v>
+      </c>
+      <c r="N8" s="31" t="n">
+        <v>4.829687595367432</v>
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
@@ -7084,17 +7168,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
-      <c r="M21" s="5" t="n"/>
-      <c r="N21" s="31" t="n"/>
+      <c r="D21" s="5" t="n">
+        <v>0.5054446859283357</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.519199366453035</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.5178086392366672</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.4954837457655661</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.511337848264892</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0.50891858524168</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>0.5717420902235882</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.5275748647375792</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>0.5119562703885332</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>0.5843122972986872</v>
+      </c>
+      <c r="N21" s="31" t="n">
+        <v>0.5073863484216871</v>
+      </c>
       <c r="O21" s="14" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -7298,17 +7404,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
-      <c r="M28" s="5" t="n"/>
-      <c r="N28" s="31" t="n"/>
+      <c r="D28" s="5" t="n">
+        <v>0.7830597621110132</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>0.8064073298678864</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0.7937104727462332</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0.7627448026242314</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>0.8009410518420114</v>
+      </c>
+      <c r="I28" s="5" t="n">
+        <v>0.7909752895896033</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>0.8419165604351599</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0.8160420765709792</v>
+      </c>
+      <c r="L28" s="5" t="n">
+        <v>0.798767023558475</v>
+      </c>
+      <c r="M28" s="5" t="n">
+        <v>0.8552598551268979</v>
+      </c>
+      <c r="N28" s="31" t="n">
+        <v>0.7923201582427839</v>
+      </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -7512,17 +7640,39 @@
           <t>BYOD-Llama (128 it.)</t>
         </is>
       </c>
-      <c r="D35" s="5" t="n"/>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="5" t="n"/>
-      <c r="L35" s="5" t="n"/>
-      <c r="M35" s="5" t="n"/>
-      <c r="N35" s="31" t="n"/>
+      <c r="D35" s="5" t="n">
+        <v>0.8727189519854217</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0.8991272440231518</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0.8846654157733219</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0.8559358721535252</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>0.8956816655050087</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>0.8853025773993753</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>0.9242696608846586</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>0.9041828997570535</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>0.8914650348851834</v>
+      </c>
+      <c r="M35" s="5" t="n">
+        <v>0.9318457286887116</v>
+      </c>
+      <c r="N35" s="31" t="n">
+        <v>0.8864252529499462</v>
+      </c>
       <c r="O35" s="14" t="inlineStr">
         <is>
           <t>LLaDA (128 it.)</t>
@@ -7639,7 +7789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B86"/>
+  <dimension ref="A1:B92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" style="33" min="1" max="1"/>
@@ -8493,90 +8643,160 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Autoregressive reference run ID</t>
+          <t>128-NFE progression run ID</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>20260923T134029.046940Z--colab-validation</t>
+          <t>20260923T201036.622289Z--colab-validation</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Autoregressive reference model</t>
+          <t>128-NFE progression completed UTC</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>meta-llama/Llama-3.1-8B-Instruct</t>
+          <t>2026-09-23T22:16:14.309989+00:00</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Autoregressive reference scored prompts</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>100</v>
+          <t>128-NFE progression source</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/validation/benchmark_runs/20260923T201036.622289Z--colab-validation/summary.json</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Autoregressive reference perplexity</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>2.638597726821899</v>
+          <t>128-NFE imported global updates</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1k, 5k, 10k, 15k, 20k, 25k, 30k, 35k, 40k, 45k, 50k</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Autoregressive reference mean Distinct-1</t>
+          <t>128-NFE scored prompts per checkpoint</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.620703125</v>
+        <v>100</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Long-run validation-loss source</t>
+          <t>128-NFE imported metrics</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/outputs/llama-3.1-8b-mask-long/metrics.jsonl</t>
+          <t>Token-weighted perplexity; mean sliding model-token Distinct-1/2/3</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Long-run validation-loss snapshot</t>
+          <t>Autoregressive reference run ID</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>steps 500--50000 in increments of 500</t>
+          <t>20260923T134029.046940Z--colab-validation</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>Autoregressive reference model</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>meta-llama/Llama-3.1-8B-Instruct</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Autoregressive reference scored prompts</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Autoregressive reference perplexity</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2.638597726821899</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Autoregressive reference mean Distinct-1</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.620703125</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Long-run validation-loss source</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>/Users/rkuiper/Library/CloudStorage/GoogleDrive-ruurd.kuiper@gmail.com/My Drive/lad-generic-results/outputs/llama-3.1-8b-mask-long/metrics.jsonl</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Long-run validation-loss snapshot</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>steps 500--50000 in increments of 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>Progression import timestamp UTC</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>2026-09-23T20:12:06.859324+00:00</t>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-09-24T05:47:36.907885+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>